<commit_message>
feat(productos): Kit de Tareas Restaurante Creativo v2.0 (477 tareas, 13 ficheros; plantillas A/B/C diferenciadas por franja/partida/perfil) — motor 2.4 + contenido propio; idempotencia 0, censo 0, gate offline 13/13
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-restaurante-creativo/01-apertura-cierre.xlsx
+++ b/astro-site/public/dl/kit-tareas-restaurante-creativo/01-apertura-cierre.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -697,9 +697,45 @@
     </row>
     <row r="15"/>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-tareas-restaurante-creativo · info@aichef.pro</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Antes de encender nada:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>▸ La primera sección de «Apertura AM» es de higiene personal y de arranque seguro: campana primero, comprobación del gas después y sólo entonces Roner, hornos, deshidratador y sopletes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>▸ Las cámaras no se «encienden» por la mañana: se COMPRUEBA que han funcionado toda la noche. Anota la lectura en la propia tarea (refrigeración 0-4 °C, congelación ≤ −18 °C, y en las de maduración también la humedad).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>▸ El cierre incluye el registro diario de jornada de la brigada: es obligatorio, se valida cada día y se conserva 4 años.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-tareas-restaurante-creativo · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -724,7 +760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -754,7 +790,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>🌅 APERTURA — EQUIPAMIENTO VANGUARDIA</t>
+          <t>🧼 APERTURA — HIGIENE PERSONAL Y ARRANQUE SEGURO</t>
         </is>
       </c>
     </row>
@@ -801,7 +837,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Encender baños térmicos / Roner / equipos sous-vide</t>
+          <t>Uniforme y calzado de trabajo limpios, delantal cambiado y pelo recogido (gorro o redecilla)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -820,7 +856,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Verificar temperatura del Roner (ajustar según prod. del día)</t>
+          <t>Sin anillos, reloj ni pulseras; uñas cortas, limpias y sin esmalte</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -839,7 +875,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Encender deshidratador y verificar bandejas en proceso</t>
+          <t>Heridas y cortes cubiertos con apósito impermeable de color visible y guante encima</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -858,12 +894,12 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Revisar fermentaciones activas: medir pH y registrar</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>I+D</t>
+          <t>Lavado de manos al entrar y en cada cambio de tarea: jabón, agua caliente y papel de un solo uso</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D9" s="11" t="n"/>
@@ -877,12 +913,12 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Verificar cámaras de maduración (temp., humedad)</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Cámara</t>
+          <t>Declarar síntomas digestivos o respiratorios: quien los tenga no manipula alimentos</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D10" s="11" t="n"/>
@@ -896,12 +932,12 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Encender Pacojet / máquina de helados (si hay producción)</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>Pastelería</t>
+          <t>Encender la campana extractora y ventilar la cocina ANTES de encender nada más</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D11" s="11" t="n"/>
@@ -915,7 +951,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Encender sifones y cargar N2O según necesidad del menú</t>
+          <t>Si la cocina tiene gas: abrir la llave general y comprobar que NO huele a gas; si huele, no enciendas nada, ventila y avisa al mantenedor</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -934,7 +970,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Verificar estado del deshidratador: texturas, tiempos restantes</t>
+          <t>Cartuchos de butano de los sopletes y cargadores de N2O: cerrados, en vertical y lejos de hornos, salamandra y focos de calor</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -947,58 +983,76 @@
       <c r="F13" s="11" t="n"/>
       <c r="G13" s="13" t="n"/>
     </row>
-    <row r="14"/>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>🌅 APERTURA — EQUIPAMIENTO VANGUARDIA</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>🔥 APERTURA — BASES Y MISE EN PLACE</t>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Zona</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>Responsable</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Hora</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Notas</t>
-        </is>
-      </c>
+      <c r="A16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Encender baños térmicos / Roner / equipos sous-vide (sólo después de la campana y del control del gas)</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Verificar stock de bases: caldos, glacés, demi-glace</t>
+          <t>Verificar temperatura del Roner (ajustar según prod. del día)</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -1013,16 +1067,16 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Verificar aceites infusionados, vinagres fermentados</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>I+D</t>
+          <t>Encender deshidratador y verificar bandejas en proceso</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D18" s="11" t="n"/>
@@ -1032,11 +1086,11 @@
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Comprobar stock de hidrocoloides y texturizantes</t>
+          <t>Revisar fermentaciones activas: medir pH y registrar</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -1051,16 +1105,16 @@
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Revisar pre-elaboraciones en curso (sous-vide 24-72h)</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Cocina</t>
+          <t>Comprobar que las cámaras de maduración han funcionado toda la noche: temperatura y humedad dentro de tus parámetros — anota la lectura: ____ °C / ____ % HR. Si hay desviación, no uses la pieza hasta valorarla</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="D20" s="11" t="n"/>
@@ -1070,16 +1124,16 @@
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Montar estaciones de partida por cada pase del menú</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>Mise en place</t>
+          <t>Comprobar que las cámaras frigoríficas y el congelador han funcionado toda la noche y registrar la temperatura (refrigeración 0-4 °C / congelación ≤ −18 °C) — anota la lectura: ____ °C. Si hay desviación, no uses el género hasta valorarlo</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="D21" s="11" t="n"/>
@@ -1089,16 +1143,16 @@
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Verificar plating bible actualizada y visible en cada pase</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>Emplatado</t>
+          <t>Encender Pacojet / máquina de helados (si hay producción)</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Pastelería</t>
         </is>
       </c>
       <c r="D22" s="11" t="n"/>
@@ -1108,11 +1162,11 @@
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Comprobar stock de microbrotes, flores comestibles</t>
+          <t>Encender sifones y cargar N2O según necesidad del menú</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1127,11 +1181,11 @@
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Verificar cortes y porciones del día (0,01g precisión)</t>
+          <t>Verificar estado del deshidratador: texturas, tiempos restantes</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1148,7 +1202,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>🍽️ APERTURA — SALA Y BRIEFING</t>
+          <t>🔥 APERTURA — BASES Y MISE EN PLACE</t>
         </is>
       </c>
     </row>
@@ -1195,12 +1249,12 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Climatización sala: temperatura, aroma, humedad</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>Sala</t>
+          <t>Verificar stock de bases: caldos, glacés, demi-glace</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D28" s="11" t="n"/>
@@ -1214,12 +1268,12 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Iluminación: verificar escenas de luz por turno</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>Sala</t>
+          <t>Verificar aceites infusionados, vinagres fermentados</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>I+D</t>
         </is>
       </c>
       <c r="D29" s="11" t="n"/>
@@ -1233,12 +1287,12 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Música ambiente: playlist seleccionada para el servicio</t>
-        </is>
-      </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>Sala</t>
+          <t>Comprobar stock de hidrocoloides y texturizantes</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>I+D</t>
         </is>
       </c>
       <c r="D30" s="11" t="n"/>
@@ -1252,12 +1306,12 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Montar mesas: mantelería, vajilla de autor, cubertería</t>
-        </is>
-      </c>
-      <c r="C31" s="17" t="inlineStr">
-        <is>
-          <t>Sala</t>
+          <t>Revisar pre-elaboraciones en curso (sous-vide 24-72h)</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D31" s="11" t="n"/>
@@ -1271,12 +1325,12 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Verificar copas de maridaje preparadas por mesa</t>
-        </is>
-      </c>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>Sumiller</t>
+          <t>Montar estaciones de partida por cada pase del menú</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Mise en place</t>
         </is>
       </c>
       <c r="D32" s="11" t="n"/>
@@ -1290,12 +1344,12 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Briefing cocina: menú del día, cambios, alérgenos reservas</t>
+          <t>Verificar plating bible actualizada y visible en cada pase</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Cocina</t>
+          <t>Emplatado</t>
         </is>
       </c>
       <c r="D33" s="11" t="n"/>
@@ -1309,12 +1363,12 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Briefing sala: storytelling de cada pase, VIPs, alérgenos</t>
-        </is>
-      </c>
-      <c r="C34" s="17" t="inlineStr">
-        <is>
-          <t>Maître</t>
+          <t>Comprobar stock de microbrotes, flores comestibles</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D34" s="11" t="n"/>
@@ -1328,12 +1382,12 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Comprobar reservas del día y mapa de sala actualizado</t>
-        </is>
-      </c>
-      <c r="C35" s="17" t="inlineStr">
-        <is>
-          <t>Maître</t>
+          <t>Verificar cortes y porciones del día (0,01g precisión)</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
         </is>
       </c>
       <c r="D35" s="11" t="n"/>
@@ -1341,58 +1395,256 @@
       <c r="F35" s="11" t="n"/>
       <c r="G35" s="13" t="n"/>
     </row>
-    <row r="36">
-      <c r="B36" s="22" t="inlineStr">
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>🍽️ APERTURA — SALA Y BRIEFING</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Climatización sala: temperatura, aroma, humedad</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>Sala</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="13" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Iluminación: verificar escenas de luz por turno</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>Sala</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Música ambiente: playlist seleccionada para el servicio</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>Sala</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Montar mesas: mantelería, vajilla de autor, cubertería</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>Sala</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Verificar copas de maridaje preparadas por mesa</t>
+        </is>
+      </c>
+      <c r="C43" s="18" t="inlineStr">
+        <is>
+          <t>Sumiller</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Briefing cocina: menú del día, cambios, alérgenos reservas</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Briefing sala: storytelling de cada pase, VIPs, alérgenos</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>Maître</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Comprobar reservas del día y mapa de sala actualizado</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>Maître</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="13" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>Tareas completadas:</t>
         </is>
       </c>
-      <c r="C36">
-        <f>COUNTIF(E6:E35,"✓")</f>
-        <v>2.0</v>
-      </c>
-      <c r="D36" t="inlineStr">
+      <c r="C47">
+        <f>COUNTIFS(B6:B46,"?*",E6:E46,"✓")-COUNTIFS(B6:B46,"Tarea",E6:E46,"✓")</f>
+        <v>0.0</v>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="E36">
-        <f>COUNTIF(B6:B35,"?*")</f>
-        <v>26.0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="E47">
+        <f>COUNTIF(B6:B46,"?*")-COUNTIF(B6:B46,"Tarea")-COUNTIF(E6:E46,"N/A")</f>
+        <v>33.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>Firma responsable: _________________  Fecha: ___/___/______</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="19" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A37:G37"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A48:G48"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A26:G26"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:G35">
+  <conditionalFormatting sqref="A6:G46">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E6="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E6 E7 E8 E9 E10 E11 E12 E13 E17 E18 E19 E20 E21 E22 E23 E24 E28 E29 E30 E31 E32 E33 E34 E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Usa ✓, ✗ o —" prompt="Marca ✓ si completada" type="list">
-      <formula1>"✓,✗,—"</formula1>
+    <dataValidation sqref="E6 E7 E8 E9 E10 E11 E12 E13 E16 E17 E18 E19 E20 E21 E22 E23 E24 E28 E29 E30 E31 E32 E33 E34 E35 E39 E40 E41 E42 E43 E44 E45 E46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." prompt="Marca ✓ si completada" type="list" errorStyle="stop">
+      <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -1415,7 +1667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1492,7 +1744,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Registrar temperaturas de todas las cámaras frigoríficas</t>
+          <t>Registrar la temperatura de todas las cámaras frigoríficas y del congelador (refrigeración 0-4 °C / congelación ≤ −18 °C) — anota la lectura: ____ °C</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -1568,7 +1820,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Etiquetar TODAS las pre-elaboraciones (fecha, hora, contenido)</t>
+          <t>Etiquetar TODAS las pre-elaboraciones (fecha, hora, contenido) y anotar la fecha límite de uso: la vida útil por familia en congelación está en la tabla del pie de «Semanales» (05-tareas-semanales-mensuales)</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -1924,7 +2176,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Registrar mermas significativas del servicio</t>
+          <t>Anotar las mermas del día (producto, cantidad y motivo): es el dato que corrige el escandallo del plato y el pedido de mañana</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
@@ -1962,7 +2214,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Activar alarma y cerrar instalaciones</t>
+          <t>Cerrar y validar el registro diario de jornada de toda la brigada (cocina y sala), con las horas reales de entrada y salida: es obligatorio y hay que conservarlo 4 años</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
@@ -1976,57 +2228,76 @@
       <c r="G32" s="13" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="22" t="inlineStr">
+      <c r="A33" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Activar alarma y cerrar instalaciones</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="13" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="22" t="inlineStr">
         <is>
           <t>Tareas completadas:</t>
         </is>
       </c>
-      <c r="C33">
-        <f>COUNTIF(E6:E32,"✓")</f>
-        <v>2.0</v>
-      </c>
-      <c r="D33" t="inlineStr">
+      <c r="C34">
+        <f>COUNTIFS(B6:B33,"?*",E6:E33,"✓")-COUNTIFS(B6:B33,"Tarea",E6:E33,"✓")</f>
+        <v>0.0</v>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="E33">
-        <f>COUNTIF(B6:B32,"?*")</f>
-        <v>23.0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>Firma responsable: _________________  Fecha: ___/___/______</t>
-        </is>
+      <c r="E34">
+        <f>COUNTIF(B6:B33,"?*")-COUNTIF(B6:B33,"Tarea")-COUNTIF(E6:E33,"N/A")</f>
+        <v>22.0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
+          <t>Firma responsable: _________________  Fecha: ___/___/______</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="A35:G35"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:G32">
+  <conditionalFormatting sqref="A6:G33">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E6="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E6 E7 E8 E9 E10 E14 E15 E16 E17 E18 E19 E20 E21 E25 E26 E27 E28 E29 E30 E31 E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Usa ✓, ✗ o —" prompt="Marca ✓ si completada" type="list">
-      <formula1>"✓,✗,—"</formula1>
+    <dataValidation sqref="E6 E7 E8 E9 E10 E14 E15 E16 E17 E18 E19 E20 E21 E25 E26 E27 E28 E29 E30 E31 E32 E33" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." prompt="Marca ✓ si completada" type="list" errorStyle="stop">
+      <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>

</xml_diff>